<commit_message>
Test manuel création bilan V3 OK
</commit_message>
<xml_diff>
--- a/Python/tests/vte/data/Evaluation-Stagiaires-Global-TEL.xlsx
+++ b/Python/tests/vte/data/Evaluation-Stagiaires-Global-TEL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\instnt\partage\FORMATIONS_C\TEL\P07-bilan-sessions-et-bilan-formation\rapports-sessions-CSV-evaluations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vt238770\Documents\_CEA\Prog\Python\tests\vte\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368A1B7E-9C8A-459A-AABF-2F8CCD93D8C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933FE12F-046C-46F0-8220-0FEE5F3CACF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TCD - Stagiaires" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="24" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -835,6 +835,12 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -848,12 +854,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1417,6 +1417,13 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <bgColor theme="9" tint="-0.249977111117893"/>
         </patternFill>
@@ -1608,13 +1615,6 @@
     <dxf>
       <alignment vertical="center"/>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -6143,7 +6143,340 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="TCD_notes_par_apprenant" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="7" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="NOM Prénom ">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="Tableau croisé dynamique3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="7" minRefreshableVersion="3" rowGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="NOM Prénom">
+  <location ref="A37:A58" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
+  <pivotFields count="17">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisPage" numFmtId="1" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="22">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="16">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="11"/>
+  </rowFields>
+  <rowItems count="21">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="4">
+    <pageField fld="5" hier="-1"/>
+    <pageField fld="7" hier="-1"/>
+    <pageField fld="3" hier="-1"/>
+    <pageField fld="14" hier="-1"/>
+  </pageFields>
+  <formats count="1">
+    <format dxfId="78">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleMedium14" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="TCD_notes" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="7" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Critères">
+  <location ref="A7:B24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+  <pivotFields count="17">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisPage" numFmtId="1" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="4"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item h="1" x="5"/>
+        <item h="1" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="16">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="13"/>
+    <field x="14"/>
+  </rowFields>
+  <rowItems count="17">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="14"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="3">
+    <pageField fld="5" hier="-1"/>
+    <pageField fld="7" hier="-1"/>
+    <pageField fld="3" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Note moyenne" fld="15" subtotal="average" baseField="14" baseItem="10" numFmtId="167"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleMedium14" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000002000000}" name="TCD_notes_par_apprenant" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="7" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="NOM Prénom ">
   <location ref="D37:U59" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>
@@ -6375,50 +6708,50 @@
     <dataField name="Note moyenne" fld="15" subtotal="average" baseField="11" baseItem="8" numFmtId="167"/>
   </dataFields>
   <formats count="54">
-    <format dxfId="118">
+    <format dxfId="119">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="117">
+    <format dxfId="118">
       <pivotArea field="13" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="116">
+    <format dxfId="117">
       <pivotArea field="14" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="115">
+    <format dxfId="116">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="114">
+    <format dxfId="115">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="113">
+    <format dxfId="114">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="0" defaultSubtotal="1"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="112">
+    <format dxfId="113">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="111">
+    <format dxfId="112">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="110">
+    <format dxfId="111">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="0" defaultSubtotal="1"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="109">
+    <format dxfId="110">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
     <format>
@@ -6433,28 +6766,28 @@
     <format>
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="108">
+    <format dxfId="109">
       <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="107">
+    <format dxfId="108">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="106">
+    <format dxfId="107">
       <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="105">
+    <format dxfId="106">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="104">
+    <format dxfId="105">
       <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="103">
+    <format dxfId="104">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="102">
+    <format dxfId="103">
       <pivotArea field="11" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="101">
+    <format dxfId="102">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6463,7 +6796,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="100">
+    <format dxfId="101">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6472,7 +6805,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="99">
+    <format dxfId="100">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6481,7 +6814,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="98">
+    <format dxfId="99">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6490,10 +6823,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="97">
+    <format dxfId="98">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="96">
+    <format dxfId="97">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6508,7 +6841,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="95">
+    <format dxfId="96">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6523,7 +6856,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="94">
+    <format dxfId="95">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6536,7 +6869,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="93">
+    <format dxfId="94">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6549,10 +6882,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="92">
+    <format dxfId="93">
       <pivotArea field="11" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="91">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6567,7 +6900,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6582,7 +6915,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="90">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6595,7 +6928,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="13" count="1" selected="0">
@@ -6608,7 +6941,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="87">
+    <format dxfId="88">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -6692,7 +7025,7 @@
     <format>
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1">
@@ -6701,7 +7034,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" offset="IV1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6710,7 +7043,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1">
@@ -6719,7 +7052,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="83">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" offset="IV1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6728,7 +7061,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1">
@@ -6737,7 +7070,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" offset="IV1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6746,7 +7079,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1">
@@ -6755,7 +7088,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" offset="IV1" fieldPosition="0">
         <references count="1">
           <reference field="13" count="1" defaultSubtotal="1">
@@ -6764,7 +7097,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" offset="IV1" fieldPosition="0"/>
     </format>
   </formats>
@@ -6777,342 +7110,15 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="Tableau croisé dynamique3" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="7" minRefreshableVersion="3" rowGrandTotals="0" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="NOM Prénom">
-  <location ref="A37:A58" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="4" colPageCount="1"/>
-  <pivotFields count="17">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField axis="axisPage" numFmtId="1" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="22">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="16">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="7"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="11"/>
-  </rowFields>
-  <rowItems count="21">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="4">
-    <pageField fld="5" hier="-1"/>
-    <pageField fld="7" hier="-1"/>
-    <pageField fld="3" hier="-1"/>
-    <pageField fld="14" hier="-1"/>
-  </pageFields>
-  <formats count="1">
-    <format dxfId="119">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="11" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleMedium14" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000001000000}" name="TCD_notes" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="7" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Critères">
-  <location ref="A7:B24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
-  <pivotFields count="17">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField axis="axisPage" numFmtId="1" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="4"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="16">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="7"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="13"/>
-    <field x="14"/>
-  </rowFields>
-  <rowItems count="17">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="14"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="3">
-    <pageField fld="5" hier="-1"/>
-    <pageField fld="7" hier="-1"/>
-    <pageField fld="3" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Note moyenne" fld="15" subtotal="average" baseField="14" baseItem="10" numFmtId="167"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleMedium14" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Stagiaires" displayName="Stagiaires" ref="A2:Q231" totalsRowShown="0" headerRowDxfId="77">
-  <autoFilter ref="A2:Q231" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="A2:Q231" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="2025"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="17">
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="N° Session" dataDxfId="76"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Formation" dataDxfId="75"/>
@@ -7483,22 +7489,22 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:U73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="60.5546875" style="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.21875" style="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="2.21875" style="28" customWidth="1"/>
-    <col min="4" max="4" width="38.44140625" style="28" customWidth="1"/>
-    <col min="5" max="19" width="9.6640625" style="28" customWidth="1"/>
+    <col min="1" max="1" width="60.5703125" style="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="2.28515625" style="28" customWidth="1"/>
+    <col min="4" max="4" width="38.42578125" style="28" customWidth="1"/>
+    <col min="5" max="19" width="9.7109375" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:2" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" s="34"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -7506,7 +7512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -7514,7 +7520,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -7522,7 +7528,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -7530,7 +7536,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -7538,7 +7544,7 @@
         <v>4.8684210526315788</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>8</v>
       </c>
@@ -7546,7 +7552,7 @@
         <v>4.7368421052631575</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>9</v>
       </c>
@@ -7554,7 +7560,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
@@ -7562,7 +7568,7 @@
         <v>4.6216216216216219</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>11</v>
       </c>
@@ -7570,7 +7576,7 @@
         <v>4.7368421052631575</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>12</v>
       </c>
@@ -7578,7 +7584,7 @@
         <v>4.666666666666667</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>13</v>
       </c>
@@ -7586,7 +7592,7 @@
         <v>4.5789473684210522</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>14</v>
       </c>
@@ -7594,7 +7600,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
@@ -7602,7 +7608,7 @@
         <v>4.5263157894736841</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>16</v>
       </c>
@@ -7610,7 +7616,7 @@
         <v>4.7894736842105265</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>17</v>
       </c>
@@ -7618,7 +7624,7 @@
         <v>4.2631578947368425</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>18</v>
       </c>
@@ -7626,7 +7632,7 @@
         <v>4.7058823529411766</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>19</v>
       </c>
@@ -7634,7 +7640,7 @@
         <v>4.7894736842105265</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>20</v>
       </c>
@@ -7642,7 +7648,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
         <v>21</v>
       </c>
@@ -7650,7 +7656,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>22</v>
       </c>
@@ -7658,7 +7664,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>23</v>
       </c>
@@ -7666,25 +7672,25 @@
         <v>4.6684782608695654</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="1:12" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="29" t="s">
+    <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:12" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="30"/>
-      <c r="D31" s="29" t="s">
+      <c r="B31" s="32"/>
+      <c r="D31" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
+      <c r="K31" s="32"/>
+      <c r="L31" s="32"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>1</v>
       </c>
@@ -7692,7 +7698,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
@@ -7706,7 +7712,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>4</v>
       </c>
@@ -7720,7 +7726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>26</v>
       </c>
@@ -7734,7 +7740,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:21" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:21" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>27</v>
       </c>
@@ -7761,48 +7767,48 @@
       <c r="T37" s="15"/>
       <c r="U37" s="15"/>
     </row>
-    <row r="38" spans="1:21" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="17" t="s">
         <v>55</v>
       </c>
       <c r="D38" s="15"/>
-      <c r="E38" s="35" t="s">
+      <c r="E38" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="F38" s="35"/>
-      <c r="G38" s="35" t="s">
+      <c r="F38" s="29"/>
+      <c r="G38" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="H38" s="35" t="s">
+      <c r="H38" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="I38" s="35"/>
-      <c r="J38" s="35"/>
-      <c r="K38" s="35"/>
-      <c r="L38" s="35" t="s">
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="29"/>
+      <c r="L38" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="M38" s="35" t="s">
+      <c r="M38" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="N38" s="35"/>
-      <c r="O38" s="35"/>
-      <c r="P38" s="35"/>
-      <c r="Q38" s="35" t="s">
+      <c r="N38" s="29"/>
+      <c r="O38" s="29"/>
+      <c r="P38" s="29"/>
+      <c r="Q38" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="R38" s="35" t="s">
+      <c r="R38" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="S38" s="35"/>
-      <c r="T38" s="35" t="s">
+      <c r="S38" s="29"/>
+      <c r="T38" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="U38" s="36" t="s">
+      <c r="U38" s="30" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:21" ht="115.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:21" ht="115.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="17" t="s">
         <v>62</v>
       </c>
@@ -7851,7 +7857,7 @@
       <c r="T39" s="13"/>
       <c r="U39" s="18"/>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
         <v>65</v>
       </c>
@@ -7904,7 +7910,7 @@
         <v>3.8888888888888888</v>
       </c>
     </row>
-    <row r="41" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="17" t="s">
         <v>67</v>
       </c>
@@ -7955,7 +7961,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
         <v>71</v>
       </c>
@@ -8006,7 +8012,7 @@
         <v>4.875</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="17" t="s">
         <v>74</v>
       </c>
@@ -8059,7 +8065,7 @@
         <v>4.666666666666667</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
         <v>80</v>
       </c>
@@ -8112,7 +8118,7 @@
         <v>4.7777777777777777</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="17" t="s">
         <v>82</v>
       </c>
@@ -8165,7 +8171,7 @@
         <v>4.5555555555555554</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="17" t="s">
         <v>83</v>
       </c>
@@ -8218,7 +8224,7 @@
         <v>4.7777777777777777</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="17" t="s">
         <v>84</v>
       </c>
@@ -8271,7 +8277,7 @@
         <v>4.7777777777777777</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="17" t="s">
         <v>86</v>
       </c>
@@ -8324,7 +8330,7 @@
         <v>4.2222222222222223</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
         <v>91</v>
       </c>
@@ -8377,7 +8383,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="17" t="s">
         <v>93</v>
       </c>
@@ -8430,7 +8436,7 @@
         <v>4.7777777777777777</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="17" t="s">
         <v>96</v>
       </c>
@@ -8483,7 +8489,7 @@
         <v>4.666666666666667</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="17" t="s">
         <v>98</v>
       </c>
@@ -8536,7 +8542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="17" t="s">
         <v>102</v>
       </c>
@@ -8589,7 +8595,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="17" t="s">
         <v>106</v>
       </c>
@@ -8648,7 +8654,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="17" t="s">
         <v>114</v>
       </c>
@@ -8707,7 +8713,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="17" t="s">
         <v>115</v>
       </c>
@@ -8766,7 +8772,7 @@
         <v>4.75</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="17" t="s">
         <v>117</v>
       </c>
@@ -8825,7 +8831,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="17" t="s">
         <v>120</v>
       </c>
@@ -8884,7 +8890,7 @@
         <v>4.25</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59"/>
       <c r="D59" s="3" t="s">
         <v>23</v>
@@ -8941,7 +8947,7 @@
         <v>4.6684782608695654</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60"/>
       <c r="D60"/>
       <c r="E60"/>
@@ -8960,7 +8966,7 @@
       <c r="R60"/>
       <c r="S60"/>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61"/>
       <c r="D61"/>
       <c r="E61"/>
@@ -8979,7 +8985,7 @@
       <c r="R61"/>
       <c r="S61"/>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62"/>
       <c r="D62"/>
       <c r="E62"/>
@@ -8998,7 +9004,7 @@
       <c r="R62"/>
       <c r="S62"/>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63"/>
       <c r="D63"/>
       <c r="E63"/>
@@ -9017,7 +9023,7 @@
       <c r="R63"/>
       <c r="S63"/>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64"/>
       <c r="D64"/>
       <c r="E64"/>
@@ -9036,7 +9042,7 @@
       <c r="R64"/>
       <c r="S64"/>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A65"/>
       <c r="D65"/>
       <c r="E65"/>
@@ -9055,7 +9061,7 @@
       <c r="R65"/>
       <c r="S65"/>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A66"/>
       <c r="D66"/>
       <c r="E66"/>
@@ -9074,7 +9080,7 @@
       <c r="R66"/>
       <c r="S66"/>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A67"/>
       <c r="D67"/>
       <c r="E67"/>
@@ -9093,7 +9099,7 @@
       <c r="R67"/>
       <c r="S67"/>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A68"/>
       <c r="D68"/>
       <c r="E68"/>
@@ -9112,7 +9118,7 @@
       <c r="R68"/>
       <c r="S68"/>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A69"/>
       <c r="D69"/>
       <c r="E69"/>
@@ -9131,7 +9137,7 @@
       <c r="R69"/>
       <c r="S69"/>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70"/>
       <c r="D70"/>
       <c r="E70"/>
@@ -9150,7 +9156,7 @@
       <c r="R70"/>
       <c r="S70"/>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71"/>
       <c r="D71"/>
       <c r="E71"/>
@@ -9169,7 +9175,7 @@
       <c r="R71"/>
       <c r="S71"/>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="D72"/>
       <c r="E72"/>
       <c r="F72"/>
@@ -9187,7 +9193,7 @@
       <c r="R72"/>
       <c r="S72"/>
     </row>
-    <row r="73" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D73"/>
       <c r="E73"/>
       <c r="F73"/>
@@ -9246,49 +9252,49 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Q231"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" style="28" customWidth="1"/>
+    <col min="1" max="1" width="31.28515625" style="28" customWidth="1"/>
     <col min="2" max="2" width="64" style="28" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="28" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="28" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="28" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.5546875" style="28" customWidth="1"/>
-    <col min="8" max="9" width="10.88671875" style="28" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" style="28" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="28" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="28" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5703125" style="28" customWidth="1"/>
+    <col min="8" max="9" width="10.85546875" style="28" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" style="28" customWidth="1"/>
     <col min="11" max="11" width="16" style="28" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="36.88671875" style="28" customWidth="1"/>
-    <col min="14" max="14" width="17.44140625" style="28" customWidth="1"/>
-    <col min="15" max="15" width="56.6640625" style="28" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.5546875" style="28" customWidth="1"/>
+    <col min="12" max="13" width="36.85546875" style="28" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" style="28" customWidth="1"/>
+    <col min="15" max="15" width="56.7109375" style="28" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.5703125" style="28" customWidth="1"/>
     <col min="17" max="17" width="104" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="34" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-    </row>
-    <row r="2" spans="1:17" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+    </row>
+    <row r="2" spans="1:17" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>36</v>
       </c>
@@ -9341,7 +9347,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>48</v>
       </c>
@@ -9392,7 +9398,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>48</v>
       </c>
@@ -9443,7 +9449,7 @@
       </c>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>48</v>
       </c>
@@ -9494,7 +9500,7 @@
       </c>
       <c r="Q5" s="10"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>48</v>
       </c>
@@ -9545,7 +9551,7 @@
       </c>
       <c r="Q6" s="10"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>48</v>
       </c>
@@ -9596,7 +9602,7 @@
       </c>
       <c r="Q7" s="10"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>48</v>
       </c>
@@ -9647,7 +9653,7 @@
       </c>
       <c r="Q8" s="10"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>48</v>
       </c>
@@ -9698,7 +9704,7 @@
       </c>
       <c r="Q9" s="10"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>48</v>
       </c>
@@ -9749,7 +9755,7 @@
       </c>
       <c r="Q10" s="10"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>48</v>
       </c>
@@ -9800,7 +9806,7 @@
       </c>
       <c r="Q11" s="10"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>48</v>
       </c>
@@ -9851,7 +9857,7 @@
       </c>
       <c r="Q12" s="10"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>48</v>
       </c>
@@ -9902,7 +9908,7 @@
       </c>
       <c r="Q13" s="10"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>48</v>
       </c>
@@ -9953,7 +9959,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>48</v>
       </c>
@@ -10004,7 +10010,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>48</v>
       </c>
@@ -10055,7 +10061,7 @@
       </c>
       <c r="Q16" s="10"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>48</v>
       </c>
@@ -10106,7 +10112,7 @@
       </c>
       <c r="Q17" s="10"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>48</v>
       </c>
@@ -10157,7 +10163,7 @@
       </c>
       <c r="Q18" s="10"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>48</v>
       </c>
@@ -10208,7 +10214,7 @@
       </c>
       <c r="Q19" s="10"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>48</v>
       </c>
@@ -10259,7 +10265,7 @@
       </c>
       <c r="Q20" s="10"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>48</v>
       </c>
@@ -10310,7 +10316,7 @@
       </c>
       <c r="Q21" s="10"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>48</v>
       </c>
@@ -10361,7 +10367,7 @@
       </c>
       <c r="Q22" s="10"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>48</v>
       </c>
@@ -10412,7 +10418,7 @@
       </c>
       <c r="Q23" s="10"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>48</v>
       </c>
@@ -10463,7 +10469,7 @@
       </c>
       <c r="Q24" s="10"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>48</v>
       </c>
@@ -10514,7 +10520,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>48</v>
       </c>
@@ -10565,7 +10571,7 @@
       </c>
       <c r="Q26" s="10"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>48</v>
       </c>
@@ -10616,7 +10622,7 @@
       </c>
       <c r="Q27" s="10"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>48</v>
       </c>
@@ -10667,7 +10673,7 @@
       </c>
       <c r="Q28" s="10"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>48</v>
       </c>
@@ -10718,7 +10724,7 @@
       </c>
       <c r="Q29" s="10"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>48</v>
       </c>
@@ -10769,7 +10775,7 @@
       </c>
       <c r="Q30" s="10"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>48</v>
       </c>
@@ -10820,7 +10826,7 @@
       </c>
       <c r="Q31" s="10"/>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>48</v>
       </c>
@@ -10871,7 +10877,7 @@
       </c>
       <c r="Q32" s="10"/>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>48</v>
       </c>
@@ -10922,7 +10928,7 @@
       </c>
       <c r="Q33" s="10"/>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>48</v>
       </c>
@@ -10973,7 +10979,7 @@
       </c>
       <c r="Q34" s="10"/>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>48</v>
       </c>
@@ -11024,7 +11030,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
         <v>48</v>
       </c>
@@ -11075,7 +11081,7 @@
       </c>
       <c r="Q36" s="10"/>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
         <v>48</v>
       </c>
@@ -11126,7 +11132,7 @@
       </c>
       <c r="Q37" s="10"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
         <v>48</v>
       </c>
@@ -11177,7 +11183,7 @@
       </c>
       <c r="Q38" s="10"/>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>48</v>
       </c>
@@ -11228,7 +11234,7 @@
       </c>
       <c r="Q39" s="10"/>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>48</v>
       </c>
@@ -11279,7 +11285,7 @@
       </c>
       <c r="Q40" s="10"/>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>48</v>
       </c>
@@ -11330,7 +11336,7 @@
       </c>
       <c r="Q41" s="10"/>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8" t="s">
         <v>48</v>
       </c>
@@ -11381,7 +11387,7 @@
       </c>
       <c r="Q42" s="10"/>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
         <v>48</v>
       </c>
@@ -11432,7 +11438,7 @@
       </c>
       <c r="Q43" s="10"/>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>48</v>
       </c>
@@ -11483,7 +11489,7 @@
       </c>
       <c r="Q44" s="10"/>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
         <v>48</v>
       </c>
@@ -11536,7 +11542,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="46" spans="1:17" ht="72" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
         <v>48</v>
       </c>
@@ -11587,7 +11593,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="47" spans="1:17" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" ht="72" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
         <v>48</v>
       </c>
@@ -11638,7 +11644,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>48</v>
       </c>
@@ -11689,7 +11695,7 @@
       </c>
       <c r="Q48" s="10"/>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
         <v>48</v>
       </c>
@@ -11740,7 +11746,7 @@
       </c>
       <c r="Q49" s="10"/>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
         <v>48</v>
       </c>
@@ -11791,7 +11797,7 @@
       </c>
       <c r="Q50" s="10"/>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>48</v>
       </c>
@@ -11842,7 +11848,7 @@
       </c>
       <c r="Q51" s="10"/>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
         <v>48</v>
       </c>
@@ -11893,7 +11899,7 @@
       </c>
       <c r="Q52" s="10"/>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
         <v>48</v>
       </c>
@@ -11944,7 +11950,7 @@
       </c>
       <c r="Q53" s="10"/>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
         <v>48</v>
       </c>
@@ -11995,7 +12001,7 @@
       </c>
       <c r="Q54" s="10"/>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>48</v>
       </c>
@@ -12046,7 +12052,7 @@
       </c>
       <c r="Q55" s="10"/>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>48</v>
       </c>
@@ -12097,7 +12103,7 @@
       </c>
       <c r="Q56" s="10"/>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
         <v>48</v>
       </c>
@@ -12148,7 +12154,7 @@
       </c>
       <c r="Q57" s="10"/>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>72</v>
       </c>
@@ -12199,7 +12205,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
         <v>72</v>
       </c>
@@ -12250,7 +12256,7 @@
       </c>
       <c r="Q59" s="10"/>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
         <v>72</v>
       </c>
@@ -12301,7 +12307,7 @@
       </c>
       <c r="Q60" s="10"/>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
         <v>72</v>
       </c>
@@ -12352,7 +12358,7 @@
       </c>
       <c r="Q61" s="10"/>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
         <v>72</v>
       </c>
@@ -12403,7 +12409,7 @@
       </c>
       <c r="Q62" s="10"/>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
         <v>72</v>
       </c>
@@ -12454,7 +12460,7 @@
       </c>
       <c r="Q63" s="10"/>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
         <v>72</v>
       </c>
@@ -12505,7 +12511,7 @@
       </c>
       <c r="Q64" s="10"/>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
         <v>72</v>
       </c>
@@ -12556,7 +12562,7 @@
       </c>
       <c r="Q65" s="10"/>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8" t="s">
         <v>72</v>
       </c>
@@ -12607,7 +12613,7 @@
       </c>
       <c r="Q66" s="10"/>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
         <v>72</v>
       </c>
@@ -12658,7 +12664,7 @@
       </c>
       <c r="Q67" s="10"/>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8" t="s">
         <v>72</v>
       </c>
@@ -12709,7 +12715,7 @@
       </c>
       <c r="Q68" s="10"/>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
         <v>77</v>
       </c>
@@ -12760,7 +12766,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
         <v>77</v>
       </c>
@@ -12811,7 +12817,7 @@
       </c>
       <c r="Q70" s="10"/>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
         <v>77</v>
       </c>
@@ -12862,7 +12868,7 @@
       </c>
       <c r="Q71" s="10"/>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8" t="s">
         <v>77</v>
       </c>
@@ -12913,7 +12919,7 @@
       </c>
       <c r="Q72" s="10"/>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
         <v>77</v>
       </c>
@@ -12964,7 +12970,7 @@
       </c>
       <c r="Q73" s="10"/>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
         <v>77</v>
       </c>
@@ -13015,7 +13021,7 @@
       </c>
       <c r="Q74" s="10"/>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
         <v>77</v>
       </c>
@@ -13066,7 +13072,7 @@
       </c>
       <c r="Q75" s="10"/>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8" t="s">
         <v>77</v>
       </c>
@@ -13117,7 +13123,7 @@
       </c>
       <c r="Q76" s="10"/>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
         <v>77</v>
       </c>
@@ -13168,7 +13174,7 @@
       </c>
       <c r="Q77" s="10"/>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="8" t="s">
         <v>77</v>
       </c>
@@ -13219,7 +13225,7 @@
       </c>
       <c r="Q78" s="10"/>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
         <v>77</v>
       </c>
@@ -13270,7 +13276,7 @@
       </c>
       <c r="Q79" s="10"/>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8" t="s">
         <v>77</v>
       </c>
@@ -13321,7 +13327,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
         <v>77</v>
       </c>
@@ -13372,7 +13378,7 @@
       </c>
       <c r="Q81" s="10"/>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
         <v>77</v>
       </c>
@@ -13423,7 +13429,7 @@
       </c>
       <c r="Q82" s="10"/>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
         <v>77</v>
       </c>
@@ -13474,7 +13480,7 @@
       </c>
       <c r="Q83" s="10"/>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8" t="s">
         <v>77</v>
       </c>
@@ -13525,7 +13531,7 @@
       </c>
       <c r="Q84" s="10"/>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
         <v>77</v>
       </c>
@@ -13576,7 +13582,7 @@
       </c>
       <c r="Q85" s="10"/>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="8" t="s">
         <v>77</v>
       </c>
@@ -13627,7 +13633,7 @@
       </c>
       <c r="Q86" s="10"/>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
         <v>77</v>
       </c>
@@ -13678,7 +13684,7 @@
       </c>
       <c r="Q87" s="10"/>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="8" t="s">
         <v>77</v>
       </c>
@@ -13729,7 +13735,7 @@
       </c>
       <c r="Q88" s="10"/>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
         <v>77</v>
       </c>
@@ -13780,7 +13786,7 @@
       </c>
       <c r="Q89" s="10"/>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8" t="s">
         <v>77</v>
       </c>
@@ -13831,7 +13837,7 @@
       </c>
       <c r="Q90" s="10"/>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
         <v>77</v>
       </c>
@@ -13882,7 +13888,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8" t="s">
         <v>77</v>
       </c>
@@ -13933,7 +13939,7 @@
       </c>
       <c r="Q92" s="10"/>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
         <v>77</v>
       </c>
@@ -13984,7 +13990,7 @@
       </c>
       <c r="Q93" s="10"/>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8" t="s">
         <v>77</v>
       </c>
@@ -14035,7 +14041,7 @@
       </c>
       <c r="Q94" s="10"/>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
         <v>77</v>
       </c>
@@ -14086,7 +14092,7 @@
       </c>
       <c r="Q95" s="10"/>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8" t="s">
         <v>77</v>
       </c>
@@ -14137,7 +14143,7 @@
       </c>
       <c r="Q96" s="10"/>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
         <v>77</v>
       </c>
@@ -14188,7 +14194,7 @@
       </c>
       <c r="Q97" s="10"/>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="8" t="s">
         <v>77</v>
       </c>
@@ -14239,7 +14245,7 @@
       </c>
       <c r="Q98" s="10"/>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
         <v>77</v>
       </c>
@@ -14290,7 +14296,7 @@
       </c>
       <c r="Q99" s="10"/>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="8" t="s">
         <v>77</v>
       </c>
@@ -14341,7 +14347,7 @@
       </c>
       <c r="Q100" s="10"/>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
         <v>77</v>
       </c>
@@ -14392,7 +14398,7 @@
       </c>
       <c r="Q101" s="10"/>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="8" t="s">
         <v>77</v>
       </c>
@@ -14443,7 +14449,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
         <v>77</v>
       </c>
@@ -14494,7 +14500,7 @@
       </c>
       <c r="Q103" s="10"/>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="8" t="s">
         <v>77</v>
       </c>
@@ -14545,7 +14551,7 @@
       </c>
       <c r="Q104" s="10"/>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
         <v>77</v>
       </c>
@@ -14596,7 +14602,7 @@
       </c>
       <c r="Q105" s="10"/>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="8" t="s">
         <v>77</v>
       </c>
@@ -14647,7 +14653,7 @@
       </c>
       <c r="Q106" s="10"/>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
         <v>77</v>
       </c>
@@ -14698,7 +14704,7 @@
       </c>
       <c r="Q107" s="10"/>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="8" t="s">
         <v>77</v>
       </c>
@@ -14749,7 +14755,7 @@
       </c>
       <c r="Q108" s="10"/>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
         <v>77</v>
       </c>
@@ -14800,7 +14806,7 @@
       </c>
       <c r="Q109" s="10"/>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="8" t="s">
         <v>77</v>
       </c>
@@ -14851,7 +14857,7 @@
       </c>
       <c r="Q110" s="10"/>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
         <v>77</v>
       </c>
@@ -14902,7 +14908,7 @@
       </c>
       <c r="Q111" s="10"/>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="8" t="s">
         <v>77</v>
       </c>
@@ -14953,7 +14959,7 @@
       </c>
       <c r="Q112" s="10"/>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
         <v>77</v>
       </c>
@@ -15004,7 +15010,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="8" t="s">
         <v>77</v>
       </c>
@@ -15055,7 +15061,7 @@
       </c>
       <c r="Q114" s="10"/>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
         <v>77</v>
       </c>
@@ -15106,7 +15112,7 @@
       </c>
       <c r="Q115" s="10"/>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="8" t="s">
         <v>77</v>
       </c>
@@ -15157,7 +15163,7 @@
       </c>
       <c r="Q116" s="10"/>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
         <v>77</v>
       </c>
@@ -15208,7 +15214,7 @@
       </c>
       <c r="Q117" s="10"/>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
         <v>77</v>
       </c>
@@ -15259,7 +15265,7 @@
       </c>
       <c r="Q118" s="10"/>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
         <v>77</v>
       </c>
@@ -15310,7 +15316,7 @@
       </c>
       <c r="Q119" s="10"/>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
         <v>77</v>
       </c>
@@ -15361,7 +15367,7 @@
       </c>
       <c r="Q120" s="10"/>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
         <v>77</v>
       </c>
@@ -15412,7 +15418,7 @@
       </c>
       <c r="Q121" s="10"/>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
         <v>77</v>
       </c>
@@ -15463,7 +15469,7 @@
       </c>
       <c r="Q122" s="10"/>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
         <v>77</v>
       </c>
@@ -15514,7 +15520,7 @@
       </c>
       <c r="Q123" s="10"/>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="8" t="s">
         <v>88</v>
       </c>
@@ -15565,7 +15571,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
         <v>88</v>
       </c>
@@ -15616,7 +15622,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
         <v>88</v>
       </c>
@@ -15667,7 +15673,7 @@
       </c>
       <c r="Q126" s="10"/>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
         <v>88</v>
       </c>
@@ -15718,7 +15724,7 @@
       </c>
       <c r="Q127" s="10"/>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="8" t="s">
         <v>88</v>
       </c>
@@ -15769,7 +15775,7 @@
       </c>
       <c r="Q128" s="10"/>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
         <v>88</v>
       </c>
@@ -15820,7 +15826,7 @@
       </c>
       <c r="Q129" s="10"/>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="8" t="s">
         <v>88</v>
       </c>
@@ -15871,7 +15877,7 @@
       </c>
       <c r="Q130" s="10"/>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
         <v>88</v>
       </c>
@@ -15922,7 +15928,7 @@
       </c>
       <c r="Q131" s="10"/>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="8" t="s">
         <v>88</v>
       </c>
@@ -15973,7 +15979,7 @@
       </c>
       <c r="Q132" s="10"/>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="8" t="s">
         <v>88</v>
       </c>
@@ -16024,7 +16030,7 @@
       </c>
       <c r="Q133" s="10"/>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="8" t="s">
         <v>88</v>
       </c>
@@ -16075,7 +16081,7 @@
       </c>
       <c r="Q134" s="10"/>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="8" t="s">
         <v>88</v>
       </c>
@@ -16126,7 +16132,7 @@
       </c>
       <c r="Q135" s="10"/>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="8" t="s">
         <v>88</v>
       </c>
@@ -16177,7 +16183,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
         <v>88</v>
       </c>
@@ -16228,7 +16234,7 @@
       </c>
       <c r="Q137" s="10"/>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="8" t="s">
         <v>88</v>
       </c>
@@ -16279,7 +16285,7 @@
       </c>
       <c r="Q138" s="10"/>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="8" t="s">
         <v>88</v>
       </c>
@@ -16330,7 +16336,7 @@
       </c>
       <c r="Q139" s="10"/>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="8" t="s">
         <v>88</v>
       </c>
@@ -16381,7 +16387,7 @@
       </c>
       <c r="Q140" s="10"/>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="8" t="s">
         <v>88</v>
       </c>
@@ -16432,7 +16438,7 @@
       </c>
       <c r="Q141" s="10"/>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="8" t="s">
         <v>88</v>
       </c>
@@ -16483,7 +16489,7 @@
       </c>
       <c r="Q142" s="10"/>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="8" t="s">
         <v>88</v>
       </c>
@@ -16534,7 +16540,7 @@
       </c>
       <c r="Q143" s="10"/>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="8" t="s">
         <v>88</v>
       </c>
@@ -16585,7 +16591,7 @@
       </c>
       <c r="Q144" s="10"/>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="8" t="s">
         <v>88</v>
       </c>
@@ -16636,7 +16642,7 @@
       </c>
       <c r="Q145" s="10"/>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="8" t="s">
         <v>88</v>
       </c>
@@ -16687,7 +16693,7 @@
       </c>
       <c r="Q146" s="10"/>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="8" t="s">
         <v>88</v>
       </c>
@@ -16738,7 +16744,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="8" t="s">
         <v>88</v>
       </c>
@@ -16789,7 +16795,7 @@
       </c>
       <c r="Q148" s="10"/>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="8" t="s">
         <v>88</v>
       </c>
@@ -16840,7 +16846,7 @@
       </c>
       <c r="Q149" s="10"/>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="8" t="s">
         <v>88</v>
       </c>
@@ -16891,7 +16897,7 @@
       </c>
       <c r="Q150" s="10"/>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="8" t="s">
         <v>88</v>
       </c>
@@ -16942,7 +16948,7 @@
       </c>
       <c r="Q151" s="10"/>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="8" t="s">
         <v>88</v>
       </c>
@@ -16993,7 +16999,7 @@
       </c>
       <c r="Q152" s="10"/>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="8" t="s">
         <v>88</v>
       </c>
@@ -17044,7 +17050,7 @@
       </c>
       <c r="Q153" s="10"/>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="8" t="s">
         <v>88</v>
       </c>
@@ -17095,7 +17101,7 @@
       </c>
       <c r="Q154" s="10"/>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="8" t="s">
         <v>88</v>
       </c>
@@ -17146,7 +17152,7 @@
       </c>
       <c r="Q155" s="10"/>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="8" t="s">
         <v>88</v>
       </c>
@@ -17197,7 +17203,7 @@
       </c>
       <c r="Q156" s="10"/>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="8" t="s">
         <v>88</v>
       </c>
@@ -17248,7 +17254,7 @@
       </c>
       <c r="Q157" s="10"/>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="8" t="s">
         <v>88</v>
       </c>
@@ -17299,7 +17305,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="8" t="s">
         <v>88</v>
       </c>
@@ -17350,7 +17356,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160" s="8" t="s">
         <v>103</v>
       </c>
@@ -17401,7 +17407,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161" s="8" t="s">
         <v>103</v>
       </c>
@@ -17454,7 +17460,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A162" s="8" t="s">
         <v>103</v>
       </c>
@@ -17507,7 +17513,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A163" s="8" t="s">
         <v>103</v>
       </c>
@@ -17560,7 +17566,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164" s="8" t="s">
         <v>103</v>
       </c>
@@ -17613,7 +17619,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165" s="8" t="s">
         <v>103</v>
       </c>
@@ -17666,7 +17672,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166" s="8" t="s">
         <v>103</v>
       </c>
@@ -17719,7 +17725,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A167" s="8" t="s">
         <v>103</v>
       </c>
@@ -17772,7 +17778,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A168" s="8" t="s">
         <v>103</v>
       </c>
@@ -17825,7 +17831,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A169" s="8" t="s">
         <v>103</v>
       </c>
@@ -17878,7 +17884,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A170" s="8" t="s">
         <v>103</v>
       </c>
@@ -17931,7 +17937,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A171" s="8" t="s">
         <v>103</v>
       </c>
@@ -17984,7 +17990,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A172" s="8" t="s">
         <v>103</v>
       </c>
@@ -18035,7 +18041,7 @@
       </c>
       <c r="Q172" s="10"/>
     </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A173" s="8" t="s">
         <v>103</v>
       </c>
@@ -18088,7 +18094,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A174" s="8" t="s">
         <v>103</v>
       </c>
@@ -18139,7 +18145,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A175" s="8" t="s">
         <v>103</v>
       </c>
@@ -18190,7 +18196,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A176" s="8" t="s">
         <v>103</v>
       </c>
@@ -18241,7 +18247,7 @@
       </c>
       <c r="Q176" s="10"/>
     </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A177" s="8" t="s">
         <v>103</v>
       </c>
@@ -18292,7 +18298,7 @@
       </c>
       <c r="Q177" s="10"/>
     </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A178" s="8" t="s">
         <v>103</v>
       </c>
@@ -18343,7 +18349,7 @@
       </c>
       <c r="Q178" s="10"/>
     </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A179" s="8" t="s">
         <v>103</v>
       </c>
@@ -18394,7 +18400,7 @@
       </c>
       <c r="Q179" s="10"/>
     </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
         <v>103</v>
       </c>
@@ -18445,7 +18451,7 @@
       </c>
       <c r="Q180" s="10"/>
     </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A181" s="8" t="s">
         <v>103</v>
       </c>
@@ -18496,7 +18502,7 @@
       </c>
       <c r="Q181" s="10"/>
     </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A182" s="8" t="s">
         <v>103</v>
       </c>
@@ -18547,7 +18553,7 @@
       </c>
       <c r="Q182" s="10"/>
     </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A183" s="8" t="s">
         <v>103</v>
       </c>
@@ -18598,7 +18604,7 @@
       </c>
       <c r="Q183" s="10"/>
     </row>
-    <row r="184" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A184" s="8" t="s">
         <v>103</v>
       </c>
@@ -18649,7 +18655,7 @@
       </c>
       <c r="Q184" s="10"/>
     </row>
-    <row r="185" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A185" s="8" t="s">
         <v>103</v>
       </c>
@@ -18700,7 +18706,7 @@
       </c>
       <c r="Q185" s="10"/>
     </row>
-    <row r="186" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A186" s="8" t="s">
         <v>103</v>
       </c>
@@ -18751,7 +18757,7 @@
       </c>
       <c r="Q186" s="10"/>
     </row>
-    <row r="187" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A187" s="8" t="s">
         <v>103</v>
       </c>
@@ -18802,7 +18808,7 @@
       </c>
       <c r="Q187" s="10"/>
     </row>
-    <row r="188" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A188" s="8" t="s">
         <v>103</v>
       </c>
@@ -18853,7 +18859,7 @@
       </c>
       <c r="Q188" s="10"/>
     </row>
-    <row r="189" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A189" s="8" t="s">
         <v>103</v>
       </c>
@@ -18904,7 +18910,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="190" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
         <v>103</v>
       </c>
@@ -18955,7 +18961,7 @@
       </c>
       <c r="Q190" s="10"/>
     </row>
-    <row r="191" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A191" s="8" t="s">
         <v>103</v>
       </c>
@@ -19006,7 +19012,7 @@
       </c>
       <c r="Q191" s="10"/>
     </row>
-    <row r="192" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A192" s="8" t="s">
         <v>103</v>
       </c>
@@ -19057,7 +19063,7 @@
       </c>
       <c r="Q192" s="10"/>
     </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" s="8" t="s">
         <v>103</v>
       </c>
@@ -19108,7 +19114,7 @@
       </c>
       <c r="Q193" s="10"/>
     </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
         <v>103</v>
       </c>
@@ -19159,7 +19165,7 @@
       </c>
       <c r="Q194" s="10"/>
     </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" s="8" t="s">
         <v>103</v>
       </c>
@@ -19210,7 +19216,7 @@
       </c>
       <c r="Q195" s="10"/>
     </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" s="8" t="s">
         <v>103</v>
       </c>
@@ -19261,7 +19267,7 @@
       </c>
       <c r="Q196" s="10"/>
     </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" s="8" t="s">
         <v>103</v>
       </c>
@@ -19312,7 +19318,7 @@
       </c>
       <c r="Q197" s="10"/>
     </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" s="8" t="s">
         <v>103</v>
       </c>
@@ -19363,7 +19369,7 @@
       </c>
       <c r="Q198" s="10"/>
     </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" s="8" t="s">
         <v>103</v>
       </c>
@@ -19414,7 +19420,7 @@
       </c>
       <c r="Q199" s="10"/>
     </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" s="8" t="s">
         <v>103</v>
       </c>
@@ -19465,7 +19471,7 @@
       </c>
       <c r="Q200" s="10"/>
     </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A201" s="8" t="s">
         <v>103</v>
       </c>
@@ -19516,7 +19522,7 @@
       </c>
       <c r="Q201" s="10"/>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A202" s="8" t="s">
         <v>103</v>
       </c>
@@ -19569,7 +19575,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A203" s="8" t="s">
         <v>103</v>
       </c>
@@ -19620,7 +19626,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A204" s="8" t="s">
         <v>103</v>
       </c>
@@ -19671,7 +19677,7 @@
       </c>
       <c r="Q204" s="10"/>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A205" s="8" t="s">
         <v>103</v>
       </c>
@@ -19722,7 +19728,7 @@
       </c>
       <c r="Q205" s="10"/>
     </row>
-    <row r="206" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A206" s="8" t="s">
         <v>103</v>
       </c>
@@ -19773,7 +19779,7 @@
       </c>
       <c r="Q206" s="10"/>
     </row>
-    <row r="207" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A207" s="8" t="s">
         <v>103</v>
       </c>
@@ -19824,7 +19830,7 @@
       </c>
       <c r="Q207" s="10"/>
     </row>
-    <row r="208" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A208" s="8" t="s">
         <v>103</v>
       </c>
@@ -19875,7 +19881,7 @@
       </c>
       <c r="Q208" s="10"/>
     </row>
-    <row r="209" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A209" s="8" t="s">
         <v>103</v>
       </c>
@@ -19926,7 +19932,7 @@
       </c>
       <c r="Q209" s="10"/>
     </row>
-    <row r="210" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A210" s="8" t="s">
         <v>103</v>
       </c>
@@ -19977,7 +19983,7 @@
       </c>
       <c r="Q210" s="10"/>
     </row>
-    <row r="211" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A211" s="8" t="s">
         <v>103</v>
       </c>
@@ -20028,7 +20034,7 @@
       </c>
       <c r="Q211" s="10"/>
     </row>
-    <row r="212" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A212" s="8" t="s">
         <v>103</v>
       </c>
@@ -20079,7 +20085,7 @@
       </c>
       <c r="Q212" s="10"/>
     </row>
-    <row r="213" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A213" s="8" t="s">
         <v>103</v>
       </c>
@@ -20130,7 +20136,7 @@
       </c>
       <c r="Q213" s="10"/>
     </row>
-    <row r="214" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A214" s="8" t="s">
         <v>103</v>
       </c>
@@ -20181,7 +20187,7 @@
       </c>
       <c r="Q214" s="10"/>
     </row>
-    <row r="215" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A215" s="8" t="s">
         <v>103</v>
       </c>
@@ -20232,7 +20238,7 @@
       </c>
       <c r="Q215" s="10"/>
     </row>
-    <row r="216" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A216" s="8" t="s">
         <v>103</v>
       </c>
@@ -20283,7 +20289,7 @@
       </c>
       <c r="Q216" s="10"/>
     </row>
-    <row r="217" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A217" s="8" t="s">
         <v>103</v>
       </c>
@@ -20334,7 +20340,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="218" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A218" s="8" t="s">
         <v>103</v>
       </c>
@@ -20385,7 +20391,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="219" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A219" s="8" t="s">
         <v>103</v>
       </c>
@@ -20436,7 +20442,7 @@
       </c>
       <c r="Q219" s="10"/>
     </row>
-    <row r="220" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A220" s="8" t="s">
         <v>103</v>
       </c>
@@ -20487,7 +20493,7 @@
       </c>
       <c r="Q220" s="10"/>
     </row>
-    <row r="221" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A221" s="8" t="s">
         <v>103</v>
       </c>
@@ -20538,7 +20544,7 @@
       </c>
       <c r="Q221" s="10"/>
     </row>
-    <row r="222" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A222" s="8" t="s">
         <v>103</v>
       </c>
@@ -20589,7 +20595,7 @@
       </c>
       <c r="Q222" s="10"/>
     </row>
-    <row r="223" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A223" s="8" t="s">
         <v>103</v>
       </c>
@@ -20640,7 +20646,7 @@
       </c>
       <c r="Q223" s="10"/>
     </row>
-    <row r="224" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A224" s="8" t="s">
         <v>103</v>
       </c>
@@ -20691,7 +20697,7 @@
       </c>
       <c r="Q224" s="10"/>
     </row>
-    <row r="225" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A225" s="8" t="s">
         <v>103</v>
       </c>
@@ -20742,7 +20748,7 @@
       </c>
       <c r="Q225" s="10"/>
     </row>
-    <row r="226" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A226" s="8" t="s">
         <v>103</v>
       </c>
@@ -20793,7 +20799,7 @@
       </c>
       <c r="Q226" s="10"/>
     </row>
-    <row r="227" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A227" s="8" t="s">
         <v>103</v>
       </c>
@@ -20844,7 +20850,7 @@
       </c>
       <c r="Q227" s="10"/>
     </row>
-    <row r="228" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A228" s="8" t="s">
         <v>103</v>
       </c>
@@ -20895,7 +20901,7 @@
       </c>
       <c r="Q228" s="10"/>
     </row>
-    <row r="229" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A229" s="8" t="s">
         <v>103</v>
       </c>
@@ -20946,7 +20952,7 @@
       </c>
       <c r="Q229" s="10"/>
     </row>
-    <row r="230" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A230" s="8" t="s">
         <v>103</v>
       </c>
@@ -20997,7 +21003,7 @@
       </c>
       <c r="Q230" s="10"/>
     </row>
-    <row r="231" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A231" s="8" t="s">
         <v>103</v>
       </c>
@@ -21079,42 +21085,42 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:AG23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" style="28" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="28" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="28" customWidth="1"/>
-    <col min="5" max="5" width="25.109375" style="28" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="28" customWidth="1"/>
-    <col min="7" max="7" width="42.6640625" style="28" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="28" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="11.6640625" style="28" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="11.6640625" style="28" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="14" max="14" width="11.6640625" style="28" customWidth="1"/>
-    <col min="15" max="15" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="16" max="16" width="11.6640625" style="28" customWidth="1"/>
-    <col min="17" max="17" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="18" max="18" width="11.6640625" style="28" customWidth="1"/>
-    <col min="19" max="19" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="20" max="20" width="11.6640625" style="28" customWidth="1"/>
-    <col min="21" max="21" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="22" width="11.6640625" style="28" customWidth="1"/>
-    <col min="23" max="23" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="24" max="24" width="11.6640625" style="28" customWidth="1"/>
-    <col min="25" max="25" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="11.6640625" style="28" customWidth="1"/>
-    <col min="27" max="27" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="28" width="11.6640625" style="28" customWidth="1"/>
-    <col min="29" max="29" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="30" max="31" width="11.6640625" style="28" customWidth="1"/>
-    <col min="32" max="32" width="11.6640625" style="28" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="38.5546875" style="28" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="28" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="28" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="28" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" style="28" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="28" customWidth="1"/>
+    <col min="7" max="7" width="42.7109375" style="28" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" style="28" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="11.7109375" style="28" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="12" width="11.7109375" style="28" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="14" max="14" width="11.7109375" style="28" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="16" max="16" width="11.7109375" style="28" customWidth="1"/>
+    <col min="17" max="17" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="18" max="18" width="11.7109375" style="28" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="20" max="20" width="11.7109375" style="28" customWidth="1"/>
+    <col min="21" max="21" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="22" width="11.7109375" style="28" customWidth="1"/>
+    <col min="23" max="23" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="24" max="24" width="11.7109375" style="28" customWidth="1"/>
+    <col min="25" max="25" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="11.7109375" style="28" customWidth="1"/>
+    <col min="27" max="27" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="28" width="11.7109375" style="28" customWidth="1"/>
+    <col min="29" max="29" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="31" width="11.7109375" style="28" customWidth="1"/>
+    <col min="32" max="32" width="11.7109375" style="28" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="38.5703125" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>43</v>
       </c>
@@ -21215,7 +21221,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>54</v>
       </c>
@@ -21284,7 +21290,7 @@
       <c r="AF2" s="11"/>
       <c r="AG2" s="11"/>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>54</v>
       </c>
@@ -21333,7 +21339,7 @@
       <c r="AF3" s="11"/>
       <c r="AG3" s="11"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>54</v>
       </c>
@@ -21400,7 +21406,7 @@
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>54</v>
       </c>
@@ -21467,7 +21473,7 @@
       <c r="AF5" s="11"/>
       <c r="AG5" s="11"/>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>54</v>
       </c>
@@ -21540,7 +21546,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>54</v>
       </c>
@@ -21609,7 +21615,7 @@
       <c r="AF7" s="11"/>
       <c r="AG7" s="11"/>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>73</v>
       </c>
@@ -21678,7 +21684,7 @@
       <c r="AF8" s="11"/>
       <c r="AG8" s="11"/>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>79</v>
       </c>
@@ -21747,7 +21753,7 @@
       <c r="AF9" s="11"/>
       <c r="AG9" s="11"/>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>79</v>
       </c>
@@ -21816,7 +21822,7 @@
       <c r="AF10" s="11"/>
       <c r="AG10" s="11"/>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>79</v>
       </c>
@@ -21885,7 +21891,7 @@
       <c r="AF11" s="11"/>
       <c r="AG11" s="11"/>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>79</v>
       </c>
@@ -21954,7 +21960,7 @@
       <c r="AF12" s="11"/>
       <c r="AG12" s="11"/>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>79</v>
       </c>
@@ -22023,7 +22029,7 @@
       <c r="AF13" s="11"/>
       <c r="AG13" s="11"/>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>90</v>
       </c>
@@ -22072,7 +22078,7 @@
       <c r="AF14" s="11"/>
       <c r="AG14" s="11"/>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>90</v>
       </c>
@@ -22141,7 +22147,7 @@
       <c r="AF15" s="11"/>
       <c r="AG15" s="11"/>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>90</v>
       </c>
@@ -22210,7 +22216,7 @@
       <c r="AF16" s="11"/>
       <c r="AG16" s="11"/>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>90</v>
       </c>
@@ -22281,7 +22287,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>90</v>
       </c>
@@ -22330,7 +22336,7 @@
       <c r="AF18" s="11"/>
       <c r="AG18" s="11"/>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>105</v>
       </c>
@@ -22431,7 +22437,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>105</v>
       </c>
@@ -22506,7 +22512,7 @@
       <c r="AF20" s="11"/>
       <c r="AG20" s="11"/>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>105</v>
       </c>
@@ -22583,7 +22589,7 @@
       </c>
       <c r="AG21" s="11"/>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>105</v>
       </c>
@@ -22660,7 +22666,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>105</v>
       </c>

</xml_diff>